<commit_message>
Add email thread documentation and update test roster
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-roster.xlsx
+++ b/test-roster.xlsx
@@ -397,11 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,6 +406,9 @@
       <c r="B1" t="str">
         <v>Manager</v>
       </c>
+      <c r="C1" t="str">
+        <v>Manager Email</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -418,6 +417,9 @@
       <c r="B2" t="str">
         <v>Alice Johnson</v>
       </c>
+      <c r="C2" t="str">
+        <v>louis.lam@dwmas.co.uk</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -426,6 +428,9 @@
       <c r="B3" t="str">
         <v>Alice Johnson</v>
       </c>
+      <c r="C3" t="str">
+        <v>louis.lam@dwmas.co.uk</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -434,6 +439,9 @@
       <c r="B4" t="str">
         <v>Alice Johnson</v>
       </c>
+      <c r="C4" t="str">
+        <v>louis.lam@dwmas.co.uk</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -442,6 +450,9 @@
       <c r="B5" t="str">
         <v>Mike Davis</v>
       </c>
+      <c r="C5" t="str">
+        <v>louislam617@gmail.com</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -450,6 +461,9 @@
       <c r="B6" t="str">
         <v>Mike Davis</v>
       </c>
+      <c r="C6" t="str">
+        <v>louislam617@gmail.com</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -458,6 +472,9 @@
       <c r="B7" t="str">
         <v>Mike Davis</v>
       </c>
+      <c r="C7" t="str">
+        <v>louislam617@gmail.com</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -466,6 +483,9 @@
       <c r="B8" t="str">
         <v>Rachel Adams</v>
       </c>
+      <c r="C8" t="str">
+        <v>louis.lam@dwmas.co.uk</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -474,10 +494,13 @@
       <c r="B9" t="str">
         <v>Rachel Adams</v>
       </c>
+      <c r="C9" t="str">
+        <v>louis.lam@dwmas.co.uk</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>